<commit_message>
Update 26-27_isik.xlsx with latest data
</commit_message>
<xml_diff>
--- a/26-27_isik.xlsx
+++ b/26-27_isik.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\IDARI\OgrenciIsleriDB\OIDB Server\CİHAN TAZEÖZ\Uygulamalar\selection_project2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2E29954-FF89-4097-86BD-76A94A64C7D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502BF97E-8896-460E-B1D0-2E2D818A95FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sayfa2" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sayfa1!$A$1:$G$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sayfa1!$A$1:$G$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="341">
   <si>
     <t>Fakülte/Yüksekokul Adı</t>
   </si>
@@ -1057,6 +1057,12 @@
   </si>
   <si>
     <t>364,8237</t>
+  </si>
+  <si>
+    <t>İNŞAAT TEKNOLOJİSİ (%50 İNDİRİMLİ)</t>
+  </si>
+  <si>
+    <t>İNŞAAT TEKNOLOJİSİ (BURSLU)</t>
   </si>
 </sst>
 </file>
@@ -1506,7 +1512,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G75"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.140625" customWidth="1"/>
@@ -1541,366 +1548,366 @@
         <v>190</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>195</v>
+        <v>233</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>196</v>
+        <v>234</v>
       </c>
       <c r="F2" s="6">
-        <v>680000</v>
+        <v>275000</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>154</v>
+        <v>119</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>197</v>
+        <v>267</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F3" s="6">
-        <v>680000</v>
+        <v>268</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>176</v>
+        <v>120</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>199</v>
+        <v>253</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>200</v>
+        <v>254</v>
       </c>
       <c r="F4" s="6">
-        <v>680000</v>
+        <v>291500</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>165</v>
+        <v>121</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>201</v>
+        <v>269</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="F5" s="6">
-        <v>732500</v>
+        <v>270</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>167</v>
+        <v>122</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>203</v>
+        <v>265</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>204</v>
+        <v>266</v>
       </c>
       <c r="F6" s="6">
-        <v>732500</v>
+        <v>583000</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>182</v>
+        <v>123</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>205</v>
+        <v>299</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>206</v>
+        <v>300</v>
       </c>
       <c r="F7" s="6">
         <v>732500</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>184</v>
+        <v>124</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>207</v>
+        <v>303</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="F8" s="6">
-        <v>732500</v>
+        <v>304</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>169</v>
+        <v>125</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>76</v>
+        <v>241</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>76</v>
+        <v>242</v>
       </c>
       <c r="F9" s="6">
-        <v>1465000</v>
+        <v>281500</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>170</v>
+        <v>126</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>209</v>
+        <v>271</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="F10" s="6">
-        <v>1465000</v>
+        <v>272</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>186</v>
+        <v>127</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>211</v>
+        <v>255</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>212</v>
+        <v>256</v>
       </c>
       <c r="F11" s="6">
-        <v>1465000</v>
+        <v>563000</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>187</v>
+        <v>128</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>213</v>
+        <v>243</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>214</v>
+        <v>244</v>
       </c>
       <c r="F12" s="6">
-        <v>1465000</v>
+        <v>281500</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>215</v>
+        <v>273</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>216</v>
+        <v>274</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>217</v>
+        <v>289</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>117</v>
+        <v>290</v>
+      </c>
+      <c r="F14" s="6">
+        <v>707500</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>166</v>
+        <v>131</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>219</v>
+        <v>305</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>220</v>
+        <v>306</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G15" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F16" s="6">
+        <v>275000</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>183</v>
+        <v>133</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>223</v>
+        <v>275</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>224</v>
+        <v>276</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>117</v>
@@ -1909,44 +1916,44 @@
         <v>192</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>185</v>
+        <v>134</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>225</v>
+        <v>291</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>117</v>
+        <v>292</v>
+      </c>
+      <c r="F18" s="6">
+        <v>707500</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>177</v>
+        <v>135</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>227</v>
+        <v>307</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>228</v>
+        <v>308</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>117</v>
@@ -1955,481 +1962,481 @@
         <v>191</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>179</v>
+        <v>136</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>229</v>
+        <v>301</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>117</v>
+        <v>302</v>
+      </c>
+      <c r="F20" s="6">
+        <v>732500</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>178</v>
+        <v>137</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>231</v>
+        <v>309</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="F21" s="6">
-        <v>680000</v>
+        <v>310</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>233</v>
+        <v>317</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>234</v>
+        <v>318</v>
       </c>
       <c r="F22" s="6">
-        <v>275000</v>
+        <v>707500</v>
       </c>
       <c r="G22" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>235</v>
+        <v>329</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="F23" s="6">
-        <v>275000</v>
+        <v>330</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>237</v>
+        <v>76</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>238</v>
+        <v>76</v>
       </c>
       <c r="F24" s="6">
-        <v>275000</v>
+        <v>1415000</v>
       </c>
       <c r="G24" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="F25" s="6">
-        <v>275000</v>
+        <v>281500</v>
       </c>
       <c r="G25" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>125</v>
+        <v>189</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>241</v>
+        <v>287</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="F26" s="6">
-        <v>281500</v>
+        <v>288</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G26" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>128</v>
+        <v>30</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>193</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>243</v>
+        <v>257</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>244</v>
+        <v>258</v>
       </c>
       <c r="F27" s="6">
-        <v>281500</v>
+        <v>707500</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>151</v>
+        <v>30</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>194</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="F28" s="6">
-        <v>281500</v>
+        <v>262</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>188</v>
+        <v>141</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="F29" s="6">
-        <v>281500</v>
+        <v>275000</v>
       </c>
       <c r="G29" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>162</v>
+        <v>142</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>249</v>
+        <v>277</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="F30" s="6">
-        <v>284000</v>
+        <v>278</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>172</v>
+        <v>143</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>251</v>
+        <v>321</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>252</v>
+        <v>322</v>
       </c>
       <c r="F31" s="6">
-        <v>284000</v>
+        <v>732500</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>120</v>
+        <v>144</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>253</v>
+        <v>331</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="F32" s="6">
-        <v>291500</v>
+        <v>332</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>255</v>
+        <v>323</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>256</v>
+        <v>324</v>
       </c>
       <c r="F33" s="6">
-        <v>563000</v>
+        <v>732500</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>193</v>
+      <c r="B34" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>257</v>
+        <v>333</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="F34" s="6">
-        <v>707500</v>
+        <v>334</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>259</v>
+        <v>325</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>260</v>
+        <v>326</v>
       </c>
       <c r="F35" s="6">
-        <v>563000</v>
+        <v>1465000</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>194</v>
+      <c r="B36" s="8" t="s">
+        <v>148</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>261</v>
+        <v>327</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>117</v>
+        <v>328</v>
+      </c>
+      <c r="F36" s="6">
+        <v>1465000</v>
       </c>
       <c r="G36" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>263</v>
+        <v>195</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>264</v>
+        <v>196</v>
       </c>
       <c r="F37" s="6">
-        <v>568000</v>
+        <v>680000</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>265</v>
+        <v>215</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F38" s="6">
-        <v>583000</v>
+        <v>216</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>119</v>
+        <v>151</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>267</v>
+        <v>245</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>117</v>
+        <v>246</v>
+      </c>
+      <c r="F39" s="6">
+        <v>281500</v>
       </c>
       <c r="G39" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>117</v>
@@ -2438,24 +2445,24 @@
         <v>192</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>117</v>
+        <v>260</v>
+      </c>
+      <c r="F41" s="6">
+        <v>563000</v>
       </c>
       <c r="G41" s="4" t="s">
         <v>192</v>
@@ -2465,20 +2472,20 @@
       <c r="A42" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B42" s="8" t="s">
-        <v>129</v>
+      <c r="B42" s="9" t="s">
+        <v>339</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>273</v>
+        <v>76</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>117</v>
+        <v>76</v>
+      </c>
+      <c r="F42" s="6">
+        <v>281500</v>
       </c>
       <c r="G42" s="4" t="s">
         <v>192</v>
@@ -2488,17 +2495,17 @@
       <c r="A43" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="8" t="s">
-        <v>133</v>
+      <c r="B43" s="9" t="s">
+        <v>340</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>275</v>
+        <v>76</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>276</v>
+        <v>76</v>
       </c>
       <c r="F43" s="6" t="s">
         <v>117</v>
@@ -2507,159 +2514,159 @@
         <v>192</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>277</v>
+        <v>197</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>117</v>
+        <v>198</v>
+      </c>
+      <c r="F44" s="6">
+        <v>680000</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>279</v>
+        <v>217</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>280</v>
+        <v>218</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>117</v>
+        <v>294</v>
+      </c>
+      <c r="F46" s="6">
+        <v>707500</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>283</v>
+        <v>311</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>284</v>
+        <v>312</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>117</v>
+        <v>296</v>
+      </c>
+      <c r="F48" s="6">
+        <v>707500</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>287</v>
+        <v>313</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>288</v>
+        <v>314</v>
       </c>
       <c r="F49" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>289</v>
+        <v>319</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>290</v>
+        <v>320</v>
       </c>
       <c r="F50" s="6">
         <v>707500</v>
@@ -2668,182 +2675,182 @@
         <v>191</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>291</v>
+        <v>337</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="F51" s="6">
-        <v>707500</v>
+        <v>338</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G51" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>293</v>
+        <v>249</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>294</v>
+        <v>250</v>
       </c>
       <c r="F52" s="6">
-        <v>707500</v>
+        <v>284000</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>295</v>
+        <v>281</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="F53" s="6">
-        <v>707500</v>
+        <v>282</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>297</v>
+        <v>263</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>298</v>
+        <v>264</v>
       </c>
       <c r="F54" s="6">
-        <v>707500</v>
+        <v>568000</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>123</v>
+        <v>165</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>299</v>
+        <v>201</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>300</v>
+        <v>202</v>
       </c>
       <c r="F55" s="6">
         <v>732500</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>136</v>
+        <v>166</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>301</v>
+        <v>219</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="F56" s="6">
+        <v>220</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F57" s="6">
         <v>732500</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B57" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>303</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="F57" s="6" t="s">
-        <v>117</v>
       </c>
       <c r="G57" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>131</v>
+        <v>168</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>305</v>
+        <v>221</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>306</v>
+        <v>222</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>117</v>
@@ -2852,389 +2859,389 @@
         <v>191</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>307</v>
+        <v>76</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="F59" s="6" t="s">
-        <v>117</v>
+        <v>76</v>
+      </c>
+      <c r="F59" s="6">
+        <v>1465000</v>
       </c>
       <c r="G59" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>137</v>
+        <v>170</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>309</v>
+        <v>209</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="F60" s="6" t="s">
-        <v>117</v>
+        <v>210</v>
+      </c>
+      <c r="F60" s="6">
+        <v>1465000</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>311</v>
+        <v>335</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>312</v>
+        <v>336</v>
       </c>
       <c r="F61" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>313</v>
+        <v>251</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>314</v>
-      </c>
-      <c r="F62" s="6" t="s">
-        <v>117</v>
+        <v>252</v>
+      </c>
+      <c r="F62" s="6">
+        <v>284000</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>315</v>
+        <v>283</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>316</v>
+        <v>284</v>
       </c>
       <c r="F63" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B64" s="8" t="s">
-        <v>138</v>
+        <v>43</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>174</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>317</v>
+        <v>239</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>318</v>
+        <v>240</v>
       </c>
       <c r="F64" s="6">
-        <v>707500</v>
+        <v>275000</v>
       </c>
       <c r="G64" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B65" s="8" t="s">
-        <v>160</v>
+        <v>43</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>175</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>319</v>
+        <v>285</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="F65" s="6">
-        <v>707500</v>
+        <v>286</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>321</v>
+        <v>199</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>322</v>
+        <v>200</v>
       </c>
       <c r="F66" s="6">
-        <v>732500</v>
+        <v>680000</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>323</v>
+        <v>227</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="F67" s="6">
-        <v>732500</v>
+        <v>228</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G67" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B68" s="8" t="s">
-        <v>140</v>
+        <v>178</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>76</v>
+        <v>231</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>76</v>
+        <v>232</v>
       </c>
       <c r="F68" s="6">
-        <v>1415000</v>
+        <v>680000</v>
       </c>
       <c r="G68" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>147</v>
+        <v>179</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>325</v>
+        <v>229</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="F69" s="6">
-        <v>1465000</v>
+        <v>230</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>117</v>
       </c>
       <c r="G69" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>148</v>
+        <v>180</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>327</v>
+        <v>297</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>328</v>
+        <v>298</v>
       </c>
       <c r="F70" s="6">
-        <v>1465000</v>
+        <v>707500</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>139</v>
+        <v>181</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>330</v>
+        <v>316</v>
       </c>
       <c r="F71" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B72" s="8" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>331</v>
+        <v>205</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>332</v>
-      </c>
-      <c r="F72" s="6" t="s">
-        <v>117</v>
+        <v>206</v>
+      </c>
+      <c r="F72" s="6">
+        <v>732500</v>
       </c>
       <c r="G72" s="4" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>146</v>
+        <v>183</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>333</v>
+        <v>223</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>334</v>
+        <v>224</v>
       </c>
       <c r="F73" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G73" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="F74" s="6">
+        <v>732500</v>
+      </c>
+      <c r="G74" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B74" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>336</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="G74" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="B75" s="8" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>337</v>
+        <v>225</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>338</v>
+        <v>226</v>
       </c>
       <c r="F75" s="6" t="s">
         <v>117</v>
@@ -3243,7 +3250,69 @@
         <v>191</v>
       </c>
     </row>
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F76" s="6">
+        <v>1465000</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F77" s="6">
+        <v>1465000</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:G77" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Meslek Yüksekokulu"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="İNŞAAT TEKNOLOJİSİ (%50 İNDİRİMLİ)"/>
+        <filter val="İNŞAAT TEKNOLOJİSİ (BURSLU)"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G77">
+      <sortCondition ref="B1:B77"/>
+    </sortState>
+  </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>

</xml_diff>